<commit_message>
feat: add orders, inventory, wishlist, cart, profile, recommendations
</commit_message>
<xml_diff>
--- a/database/ProductRecommendations.xlsx
+++ b/database/ProductRecommendations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dineb\ai-ecommerce-platform\database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9BAEAB9D-53B6-4138-9C31-15D1795C870A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E81A061-404E-4AEC-AF60-3D6B540586D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{CF2B3566-E44C-4B8C-86F0-AF3FD248DCF6}"/>
   </bookViews>
@@ -66,9 +66,6 @@
     <t>Chair,Laptop Stand</t>
   </si>
   <si>
-    <t>Laptop</t>
-  </si>
-  <si>
     <t>Mouse,Keyboard,Laptop Bag</t>
   </si>
   <si>
@@ -90,9 +87,6 @@
     <t>Bedsheet,Blanket</t>
   </si>
   <si>
-    <t>Phone</t>
-  </si>
-  <si>
     <t>Earbuds,Charger</t>
   </si>
   <si>
@@ -100,6 +94,12 @@
   </si>
   <si>
     <t>Tripod,Memory Card</t>
+  </si>
+  <si>
+    <t>Lenovo V15 G4 AMD Athlon Silver 7120U Laptop</t>
+  </si>
+  <si>
+    <t>REDMI A7 Pro 5G</t>
   </si>
 </sst>
 </file>
@@ -512,52 +512,52 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>12</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>14</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>16</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>